<commit_message>
feat: advance YourTube 2.0 Atlas features and QA
</commit_message>
<xml_diff>
--- a/outputs/01a0e3e8-d9b4-7433-af76-646a3e6c8cf2/YourTube_2.0_Requirements_Tracker.xlsx
+++ b/outputs/01a0e3e8-d9b4-7433-af76-646a3e6c8cf2/YourTube_2.0_Requirements_Tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re52a5383ad6d4704"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R82e820bcfcac44f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R09e880d0e6014e6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R86fa32cc437b4183"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -271,7 +271,7 @@
         <x:color rgb="FF145C38"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF3E5"/>
         </x:patternFill>
       </x:fill>
@@ -282,7 +282,7 @@
         <x:color rgb="FF246444"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF5ED"/>
         </x:patternFill>
       </x:fill>
@@ -293,7 +293,7 @@
         <x:color rgb="FF855A10"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D6"/>
         </x:patternFill>
       </x:fill>
@@ -304,7 +304,7 @@
         <x:color rgb="FF8B4C18"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE9D8"/>
         </x:patternFill>
       </x:fill>
@@ -315,7 +315,7 @@
         <x:color rgb="FF375B86"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F1FC"/>
         </x:patternFill>
       </x:fill>
@@ -326,7 +326,7 @@
         <x:color rgb="FF8E3540"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFBE9EA"/>
         </x:patternFill>
       </x:fill>
@@ -601,7 +601,7 @@
         <x:v>Room media</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>Three-browser media, sharing and recording need live review. The user will test Mac camera/mic.</x:v>
+        <x:v>Room browser QA on 4 Oct 2026 verified seven items; six still need physical-device or native-picker checks. The user will test Mac camera/mic.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -622,7 +622,7 @@
       </x:c>
       <x:c r="B11" s="11" t="n">
         <x:f>COUNTIF(Tracker!$E$5:$E$91,A11)</x:f>
-        <x:v>0</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -640,7 +640,7 @@
       </x:c>
       <x:c r="B13" s="11" t="n">
         <x:f>COUNTIF(Tracker!$E$5:$E$91,A13)</x:f>
-        <x:v>13</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -704,7 +704,7 @@
         <x:v>2 · Room device review</x:v>
       </x:c>
       <x:c r="B21" s="8" t="str">
-        <x:v>Test three-browser media, device controls, screen sharing and recording; user handles Mac camera/mic.</x:v>
+        <x:v>Finish physical camera/mic, mobile front/rear, native screen picker and constrained-network checks; investigate the intermittent third video feed.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="40" customHeight="1">
@@ -740,7 +740,7 @@
         <x:v>Evidence date</x:v>
       </x:c>
       <x:c r="B26" s="8" t="str">
-        <x:v>VidCircle tracker: 25 Sep 2026. YourTube 2.0 migration review: 1 Oct 2026. Tests were not rerun to create this workbook.</x:v>
+        <x:v>VidCircle tracker: 25 Sep 2026. YourTube 2.0 migration review: 1 Oct 2026. Room browser QA: 4 Oct 2026. Other journeys were not rerun for this update.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="40" customHeight="1">
@@ -1418,7 +1418,7 @@
         <x:v>IST daily reset works; monthly quota and reset are missing.</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="40" customHeight="1">
+    <x:row r="35" ht="67" customHeight="1">
       <x:c r="A35" s="17" t="str">
         <x:v>V-01</x:v>
       </x:c>
@@ -1435,7 +1435,7 @@
         <x:v>Needs live QA</x:v>
       </x:c>
       <x:c r="F35" s="8" t="str">
-        <x:v>Confirm real audio/video exchange in three signed-in browsers.</x:v>
+        <x:v>Three separate Chrome/Edge/Chrome browsers decoded synthetic video and had live audio tracks on 4 Oct. One earlier third-feed decode timed out; repeat with physical camera/mic on separate devices.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="40" customHeight="1">
@@ -1458,7 +1458,7 @@
         <x:v>Room creation/signalling is present; multi-browser review pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="40" customHeight="1">
+    <x:row r="37" ht="67" customHeight="1">
       <x:c r="A37" s="17" t="str">
         <x:v>V-03</x:v>
       </x:c>
@@ -1475,10 +1475,10 @@
         <x:v>Needs live QA</x:v>
       </x:c>
       <x:c r="F37" s="8" t="str">
-        <x:v>Test microphone and camera controls with real device permissions.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="40" customHeight="1">
+        <x:v>Mic and camera controls passed with synthetic devices in three browsers on 4 Oct. Confirm with real camera/mic permissions and observable audio/video on physical devices.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="67" customHeight="1">
       <x:c r="A38" s="17" t="str">
         <x:v>V-04</x:v>
       </x:c>
@@ -1495,10 +1495,10 @@
         <x:v>Needs live QA</x:v>
       </x:c>
       <x:c r="F38" s="8" t="str">
-        <x:v>Test device switching, including mobile front/rear cameras.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="40" customHeight="1">
+        <x:v>Desktop synthetic camera and mic switching passed on 4 Oct. Physical mobile front/rear camera switching remains to be tested.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="67" customHeight="1">
       <x:c r="A39" s="17" t="str">
         <x:v>V-05</x:v>
       </x:c>
@@ -1515,10 +1515,10 @@
         <x:v>Needs live QA</x:v>
       </x:c>
       <x:c r="F39" s="8" t="str">
-        <x:v>Test screen sharing and the remote participant view.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="40" customHeight="1">
+        <x:v>Synthetic screen source reached a remote viewer on 4 Oct. Confirm the native browser/OS screen picker and shared screen on another physical device.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="57" customHeight="1">
       <x:c r="A40" s="17" t="str">
         <x:v>V-06</x:v>
       </x:c>
@@ -1532,13 +1532,13 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="E40" s="25" t="str">
-        <x:v>Needs live QA</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F40" s="8" t="str">
-        <x:v>Test leave/end and participant state in a three-browser room.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="40" customHeight="1">
+        <x:v>Verified 4 Oct 2026: three signed-in browsers showed participants and raised hands; leave/rejoin and host end reached all clients.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="57" customHeight="1">
       <x:c r="A41" s="17" t="str">
         <x:v>V-07</x:v>
       </x:c>
@@ -1552,13 +1552,13 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="E41" s="25" t="str">
-        <x:v>Needs live QA</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F41" s="8" t="str">
-        <x:v>Test chat, emojis and small file exchange across browsers.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="40" customHeight="1">
+        <x:v>Verified 4 Oct 2026: emoji chat and a small file reached another browser; received file bytes matched the upload.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="57" customHeight="1">
       <x:c r="A42" s="17" t="str">
         <x:v>V-08</x:v>
       </x:c>
@@ -1572,13 +1572,13 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="E42" s="25" t="str">
-        <x:v>Needs live QA</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F42" s="8" t="str">
-        <x:v>Check live speaking, connection, microphone, camera and timer states.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="40" customHeight="1">
+        <x:v>Verified 4 Oct 2026: name, mic/camera, speaking, connection and call-duration indicators responded across browsers using synthetic media.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="57" customHeight="1">
       <x:c r="A43" s="17" t="str">
         <x:v>V-09</x:v>
       </x:c>
@@ -1592,13 +1592,13 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="E43" s="25" t="str">
-        <x:v>Needs live QA</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F43" s="8" t="str">
-        <x:v>Check host mute, remove and lock controls with real participants.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="40" customHeight="1">
+        <x:v>Verified 4 Oct 2026: host locked the room, muted a participant and removed them; guest controls stayed restricted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="57" customHeight="1">
       <x:c r="A44" s="17" t="str">
         <x:v>V-10</x:v>
       </x:c>
@@ -1612,13 +1612,13 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="E44" s="25" t="str">
-        <x:v>Needs live QA</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F44" s="8" t="str">
-        <x:v>Check co-host, chat and screen-sharing permissions across browsers.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="40" customHeight="1">
+        <x:v>Verified 4 Oct 2026: host assigned co-host and tested chat and screen-share permissions across signed-in browsers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="57" customHeight="1">
       <x:c r="A45" s="17" t="str">
         <x:v>V-11</x:v>
       </x:c>
@@ -1632,13 +1632,13 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="E45" s="25" t="str">
-        <x:v>Needs live QA</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F45" s="8" t="str">
-        <x:v>Record as host, then download and play the local recording.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="40" customHeight="1">
+        <x:v>Verified 4 Oct 2026: host-only recording created a 119,957-byte WebM; another browser showed recording status and the saved file played.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="57" customHeight="1">
       <x:c r="A46" s="17" t="str">
         <x:v>V-12</x:v>
       </x:c>
@@ -1652,13 +1652,13 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="E46" s="25" t="str">
-        <x:v>Needs live QA</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="F46" s="8" t="str">
-        <x:v>Test interruption recovery and browser refresh/rejoin.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="40" customHeight="1">
+        <x:v>Verified 4 Oct 2026: browser refresh/rejoin and simulated network offline/online recovery completed in the three-browser room.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="67" customHeight="1">
       <x:c r="A47" s="17" t="str">
         <x:v>V-13</x:v>
       </x:c>
@@ -1675,10 +1675,10 @@
         <x:v>Needs live QA</x:v>
       </x:c>
       <x:c r="F47" s="8" t="str">
-        <x:v>Test permission denial on a device; Mac camera/mic testing stays with the user.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="40" customHeight="1">
+        <x:v>Simulated camera/mic permission denial fell back to joining without media on 4 Oct. Confirm actual device denial; Mac camera/mic test remains with the user.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="67" customHeight="1">
       <x:c r="A48" s="17" t="str">
         <x:v>V-14</x:v>
       </x:c>
@@ -1695,7 +1695,7 @@
         <x:v>Needs live QA</x:v>
       </x:c>
       <x:c r="F48" s="8" t="str">
-        <x:v>Check noise and low-bandwidth controls with media, plus the participant cap.</x:v>
+        <x:v>Synthetic noise-suppression and low-bandwidth controls plus the four-person cap passed on 4 Oct. Confirm with real microphone/video and constrained network.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="40" customHeight="1">
@@ -2574,7 +2574,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5e7b5c737bb44c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra338430db0204457"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>